<commit_message>
Show co-authors (author2) on For sales titles
Parse author2/author2En and bios from the Titles sheet, list both
names as links on cards and detail pages, and include each person on
their own author page when a title has two credited authors.
</commit_message>
<xml_diff>
--- a/sheets/LENA-For-Sales-Titles.xlsx
+++ b/sheets/LENA-For-Sales-Titles.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,27 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -122,6 +139,56 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>LENA</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>저자1 한글</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>저자1 영문</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>저자2(공저) 한글 — 같은 책에 2명일 때</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>저자2(공저) 영문</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>저자1 소개 영문</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>저자1 소개 한글</t>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <t>저자2 소개 영문</t>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <t>저자2 소개 한글</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -450,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,10 +723,103 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>본문 미리보기: Titles 시트 preview1~preview4 열에 Drive 이미지 링크(뷰어 공개)를 넣으면 상세 표지 아래에 표시됩니다. 클릭 시 크게 봅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>■ 저자 2열 · 저자소개 (웹 클릭 연동)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>• author = 저자 한글 이름 (예: 김성효)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>• authorEn = 저자 영문 이름 (예: Seonghyo Kim)  ← 반드시 별도 열</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>• authorBio = 저자소개 영문 / authorBioKo = 저자소개 한글</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>• 사이트: 도서 카드·상세의 저자 이름 클릭 → /export/author/…</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>• 저자 목록: /export/authors</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>• 같은 저자는 책마다 author·authorEn 철자를 동일하게 맞출 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>■ 공저자 2명 (같은 책)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>• 한 셀에 "A, B" 로 합치지 말 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>• author / authorEn = 저자 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>• author2 / author2En = 저자 2 (추가 열)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>• authorBio* = 저자1 소개, authorBio2* = 저자2 소개</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• 웹: 각 이름을 따로 클릭 → 각자 저자소개 페이지</t>
         </is>
       </c>
     </row>
@@ -677,8 +837,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI8"/>
+  <dimension ref="A1:AM8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -696,162 +862,182 @@
           <t>titleKo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>author</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>authorEn</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>author2</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>author2En</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>publisher</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>publisherEn</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>format</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>rightsNote</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rightsNoteKo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>territories</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>territoriesKo</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rightsSold</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rightsSoldKo</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>pages</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>pubYear</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>coverCopy</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>coverCopyKo</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>synopsis</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>synopsisKo</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>authorBio</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>authorBioKo</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>authorBio2</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>authorBio2Ko</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
         <is>
           <t>color1</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>color2</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>featured</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>new</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>cover</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>preview1</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>preview2</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>preview3</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>preview4</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>published</t>
         </is>
@@ -883,128 +1069,128 @@
           <t>Seonghyo Kim</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>practical</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>빅피시</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Big Fish</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>print, ebook</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>World rights available (Taiwan licensed)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>세계 판권 가능 (대만 계약 완료)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Taiwan licensed · other territories available</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>대만 계약 · 기타 지역 가능</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Traditional Chinese</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>번체 중국어</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>268</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>2024</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Adult / Education professionals</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>36 scripts for facing parents with confidence · Mentor to hundreds of thousands of Korean teachers · 27 years of classroom know-how · Seonghyo-ssaem's Teacher Mentoring series</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>당당하게 학부모와 마주하기 위한 민원 대응법 36 · 대한민국 45만 교사들의 멘토 · 27년 차 현직 교사 노하우 · 성효 쌤의 교사 멘토링 1</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>A practical guide for teachers on parent communication and complaint handling—36 field-tested response scripts drawn from real classroom and school-gate situations.</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>교육 현장의 실제 사례를 바탕으로, 상처받지 않으면서도 나를 지키는 교사의 말과 태도를 정리한 실전 가이드.</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>Seonghyo Kim is a bestselling author and 29-year educator who lectures and consults for students, parents, and teachers.</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>학생·학부모·교사를 대상으로 강연과 상담을 하는 베스트셀러 작가이자 29년 차 교육자.</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>#7ec8d4</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>#2a9d8f</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>/covers/teacher-communication-skills.png</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1036,123 +1222,123 @@
           <t>Juyoung Jung</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>practical</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>한경비피</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>KED&amp;BP</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>print, ebook</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>World rights available (selected territories sold)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>세계 판권 가능 (일부 지역 계약 완료)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Vietnam licensed · other territories available</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>베트남 계약 · 기타 지역 가능</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Vietnamese</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>베트남어</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>272</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>2021</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Adult / YA</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Study habits and mindset from Harvard's top performers</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>하버드 상위 1%가 지키는 공부와 태도의 비밀</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Study habits and mindset insights from high-achieving Harvard students.</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>하버드 상위권 학생들의 학습 습관과 마인드셋을 정리한 자기계발·학습법 논픽션.</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Juyoung Jung writes on learning habits, mindset, and high-performance study culture.</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>정주영은 학습 습관과 마인드셋, 성과를 내는 공부 문화를 다루는 저자다.</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>#a4161a</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>#660708</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1184,113 +1370,113 @@
           <t>Sample Korean Author</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>fiction</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>한국 출판사</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Korean Publisher</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>print, ebook</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>World English &amp; other languages available</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>영어 포함 세계 판권 가능</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>All territories available</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>전 지역 가능</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>220</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>2025</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Adult / YA</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Classic Korean tales, retold for today's readers</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>오늘을 사는 우리를 위한, 다시 쓰는 한국 설화</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Classic Korean tales retold for a global readership.</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>한국 고전 설화를 세계 독자를 위해 다시 쓴 작품.</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>A Korean fiction writer reworking classic folklore.</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>한국 고전 설화를 현대적으로 다시 쓰는 소설가.</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>#9b2226</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>#ae2012</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1322,113 +1508,113 @@
           <t>Sample Author</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>nonfiction</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>한국 출판사</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Korean Publisher</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>print</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>World rights available</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>세계 판권 가능</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>All territories available</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>전 지역 가능</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>208</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>2024</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Adult</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Quiet cafés, side streets, and the softer side of Seoul</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>카페와 골목에서 만나는, 서울의 고요한 시간</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>A lyrical guide to the city's quieter corners.</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>카페와 골목, 일상의 리듬을 담은 서울 에세이.</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>An essayist exploring everyday Seoul.</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>서울의 카페와 골목, 일상 리듬을 에세이로 담아내는 작가.</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>#264653</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>#2a9d8f</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AM5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1460,113 +1646,113 @@
           <t>Sample Illustrator</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>picturebook</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>한국 아동 출판사</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Korean Children's House</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>print</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>World rights available · co-edition welcome</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>세계 판권 가능 · 공동판형 환영</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>All territories available</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>전 지역 가능</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>36</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>2025</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>3–7</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Courage, friendship, and a dream bigger than the mountain</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>용기와 우정, 산을 넘는 작은 호랑이의 큰 꿈</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>A warm picture book about courage, friendship, and dreaming beyond the mountain.</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>용기와 우정, 산을 넘는 꿈을 그린 따뜻한 그림책.</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>A Korean picture-book creator.</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>용기와 우정, 성장의 이야기를 그리는 그림책 작가.</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>#e76f51</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>#f4a261</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1598,113 +1784,113 @@
           <t>Sample Author</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>business</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>한국 출판사</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Korean Publisher</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>print, ebook</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>World rights available</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>세계 판권 가능</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>All territories available</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>전 지역 가능</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>256</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>2023</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Adult</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>What kimchi teaches about markets, brands, and resilience</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>김치 한 포기에 담긴 시장·브랜드·회복탄력성 이야기</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>What Korean food culture teaches about markets, branding, and resilience.</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>한식 문화에서 읽는 시장·브랜딩·회복탄력성.</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>A nonfiction writer on Korean food culture, markets, and branding.</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>한식 문화와 시장·브랜딩을 연결해 쓰는 논픽션 저자.</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>#bc4749</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>#6a040f</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1736,113 +1922,113 @@
           <t>Sample Author</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>practical</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>한국 출판사</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Korean Publisher</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Korea</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>print, ebook, audio</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>World rights available</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>세계 판권 가능</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>All territories available</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>전 지역 가능</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>160</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>2025</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Adult</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Sixty one-minute mindfulness practices for a fast city</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>바쁜 서울을 위한 마음챙김 1분 × 60</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>Sixty tiny practices for busy lives—born in one of the world's fastest cities.</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>바쁜 도시를 위한 아주 짧은 마음챙김 60.</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>A wellness writer offering short, practical mindfulness practices.</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>바쁜 도시 일상을 위한 짧은 마음챙김 실천을 전하는 웰니스 저자.</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>#40916c</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>#1b4332</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AF8" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AG8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AM8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1851,6 +2037,7 @@
   </sheetData>
   <autoFilter ref="A1:AE8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2112,7 +2299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2171,7 +2358,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>저자(한글)</t>
+          <t>저자1(한글)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>공저 시 첫 번째 저자</t>
         </is>
       </c>
     </row>
@@ -2183,9 +2375,10 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>저자(영문)</t>
-        </is>
-      </c>
+          <t>저자1(영문)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2411,9 +2604,10 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>저자소개(EN)</t>
-        </is>
-      </c>
+          <t>저자1소개(EN)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2423,9 +2617,10 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>저자소개(KO)</t>
-        </is>
-      </c>
+          <t>저자1소개(KO)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2498,6 +2693,62 @@
           <t>공개(published)</t>
         </is>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>author2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>저자2(한글)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>같은 책 두 번째 저자(공저)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>author2En</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>저자2(영문)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>authorBio2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>저자2소개(EN)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>authorBio2Ko</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>저자2소개(KO)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>